<commit_message>
Add FreeCAD project files and update MQTT management
- Added new FreeCAD project files: ELS_project.FCStd, button.FCStd, encoder2.FCStd, and nextion_simp.FCStd along with their backup versions.
- Refactored MQTT management in mqtt_manager.h and mqtt_manager.cpp:
  - Removed legacy task creation function and replaced it with a non-blocking service tick function.
  - Improved connection handling and initialization logic.
  - Updated reconnect interval to 3000 ms.
  - Enhanced command subscription handling using an array.
- Updated UI task to call mqttServiceTick regularly.
- Adjusted update rate to 3125 Hz for optimal performance.
- Removed MQTT task creation from setup in main.cpp.
- Updated MQTT GUI application to support new callback API version.
</commit_message>
<xml_diff>
--- a/SW/ESP_ELS/tools/Book3 (version 1).xlsx
+++ b/SW/ESP_ELS/tools/Book3 (version 1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jn.safe4\Documents\PlatformIO\Projects\Dreimaskin_ELS\SW\ESP_ELS\tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AE0F6FD-8617-4AE1-8D3A-24AB66443916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDABB93E-A06F-440D-99BC-CCE8DA0FD32B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="3585" windowWidth="29040" windowHeight="17520" xr2:uid="{F3ED2C2D-2482-46EE-8404-115CC90F6E33}"/>
   </bookViews>
@@ -23,7 +23,6 @@
     <definedName name="RPS">Sheet1!$M$9</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -585,7 +584,7 @@
       </c>
       <c r="Y7">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>480</v>
+        <v>624</v>
       </c>
     </row>
     <row r="8" spans="9:25" x14ac:dyDescent="0.25">
@@ -594,14 +593,14 @@
       </c>
       <c r="J8">
         <f>64/(J13)</f>
-        <v>192000</v>
+        <v>249600</v>
       </c>
       <c r="L8" t="s">
         <v>4</v>
       </c>
       <c r="M8">
         <f>1/MAXHz</f>
-        <v>5.2083333333333332E-6</v>
+        <v>4.0064102564102564E-6</v>
       </c>
       <c r="S8">
         <v>2</v>
@@ -623,7 +622,7 @@
       </c>
       <c r="Y8">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>240</v>
+        <v>312</v>
       </c>
     </row>
     <row r="9" spans="9:25" x14ac:dyDescent="0.25">
@@ -660,7 +659,7 @@
       </c>
       <c r="Y9">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>192</v>
+        <v>249.6</v>
       </c>
     </row>
     <row r="10" spans="9:25" x14ac:dyDescent="0.25">
@@ -669,7 +668,7 @@
       </c>
       <c r="M10">
         <f>MAXHz/RPS</f>
-        <v>5120</v>
+        <v>6656</v>
       </c>
       <c r="S10">
         <v>3</v>
@@ -691,7 +690,7 @@
       </c>
       <c r="Y10">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>120</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" spans="9:25" x14ac:dyDescent="0.25">
@@ -721,7 +720,7 @@
       </c>
       <c r="Y11">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>96</v>
+        <v>124.8</v>
       </c>
     </row>
     <row r="12" spans="9:25" x14ac:dyDescent="0.25">
@@ -729,7 +728,7 @@
         <v>17</v>
       </c>
       <c r="J12" s="1">
-        <v>3000</v>
+        <v>3900</v>
       </c>
       <c r="L12" t="s">
         <v>18</v>
@@ -758,7 +757,7 @@
       </c>
       <c r="Y12">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>60</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="9:25" x14ac:dyDescent="0.25">
@@ -767,7 +766,7 @@
       </c>
       <c r="J13">
         <f>1/J12</f>
-        <v>3.3333333333333332E-4</v>
+        <v>2.5641025641025641E-4</v>
       </c>
       <c r="S13">
         <v>11</v>
@@ -789,7 +788,7 @@
       </c>
       <c r="Y13">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>48</v>
+        <v>62.4</v>
       </c>
     </row>
     <row r="14" spans="9:25" x14ac:dyDescent="0.25">
@@ -820,21 +819,21 @@
       </c>
       <c r="Y14">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>38.4</v>
+        <v>49.92</v>
       </c>
     </row>
     <row r="15" spans="9:25" x14ac:dyDescent="0.25">
       <c r="M15">
         <f>INDEX(Table1[idx],MATCH(max_pulses_pr_rev,Table1[steps/rev],1))</f>
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="N15">
         <f>INDEX(Table1[steps/rev],MATCH(M15,Table1[idx],0))</f>
-        <v>5000</v>
+        <v>6400</v>
       </c>
       <c r="O15">
         <f>N15*RPS</f>
-        <v>187500</v>
+        <v>240000</v>
       </c>
       <c r="S15">
         <v>5</v>
@@ -856,7 +855,7 @@
       </c>
       <c r="Y15">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>30</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="9:25" x14ac:dyDescent="0.25">
@@ -880,7 +879,7 @@
       </c>
       <c r="Y16">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>24</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="17" spans="9:25" x14ac:dyDescent="0.25">
@@ -904,7 +903,7 @@
       </c>
       <c r="Y17">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>19.2</v>
+        <v>24.96</v>
       </c>
     </row>
     <row r="18" spans="9:25" x14ac:dyDescent="0.25">
@@ -928,7 +927,7 @@
       </c>
       <c r="Y18">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>15</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="19" spans="9:25" x14ac:dyDescent="0.25">
@@ -952,7 +951,7 @@
       </c>
       <c r="Y19">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>9.6</v>
+        <v>12.48</v>
       </c>
     </row>
     <row r="20" spans="9:25" x14ac:dyDescent="0.25">
@@ -976,7 +975,7 @@
       </c>
       <c r="Y20">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>7.5</v>
+        <v>9.75</v>
       </c>
     </row>
     <row r="21" spans="9:25" x14ac:dyDescent="0.25">
@@ -1000,7 +999,7 @@
       </c>
       <c r="Y21">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>4.8</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="22" spans="9:25" x14ac:dyDescent="0.25">
@@ -1024,7 +1023,7 @@
       </c>
       <c r="Y22">
         <f>MAXHz/Table1[[#This Row],[steps/rev]]</f>
-        <v>3.75</v>
+        <v>4.875</v>
       </c>
     </row>
     <row r="27" spans="9:25" x14ac:dyDescent="0.25">

</xml_diff>